<commit_message>
Stop reporting occupancy of 6000%
The Erlang curve gives a line per agent count, and below the offered load
it showed a service level of 0.0% beside an occupancy of 6000%, then
3000%, then 2000%, down sixty rows. It is load divided by agents, so it
is arithmetic, but it is not a number: below the offered load the queue
never clears, so there is no steady state to be occupied in.

Service level and average speed of answer both already blank themselves
there. Occupancy was the one column that did not, and it is the one a
reader scans, because it is the number that decides whether a roster is
humane. Now it matches its neighbours.

Found by reading the sheet rather than by any check — 680 verify checks,
38/38 charts, 114 visual and 200 mutants all pass with 6000% on the page,
because every one of them asks whether a number is computed correctly and
none asks whether it means anything.

Also folds the visual pass into the v3.3 notes.
</commit_message>
<xml_diff>
--- a/templates/17-control-plan.xlsx
+++ b/templates/17-control-plan.xlsx
@@ -261,7 +261,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -501,6 +501,9 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1996,7 +1999,7 @@
         <f>COUNTIF($P$10:$P$27,LEFT(A39,1)&amp;"*")</f>
         <v/>
       </c>
-      <c r="C39" s="81" t="inlineStr">
+      <c r="C39" s="82" t="inlineStr">
         <is>
           <t>Strongest of all: the failure cannot happen because the step is gone. Retiring the manual adjustment queue counts here; a better checklist does not.</t>
         </is>
@@ -2012,7 +2015,7 @@
         <f>COUNTIF($P$10:$P$27,LEFT(A40,1)&amp;"*")</f>
         <v/>
       </c>
-      <c r="C40" s="81" t="inlineStr">
+      <c r="C40" s="82" t="inlineStr">
         <is>
           <t>The system will not permit the failure — a ticket that cannot be closed while an adjustment is still in flight. Survives attrition, busy weeks and everyone forgetting.</t>
         </is>
@@ -2028,7 +2031,7 @@
         <f>COUNTIF($P$10:$P$27,LEFT(A41,1)&amp;"*")</f>
         <v/>
       </c>
-      <c r="C41" s="81" t="inlineStr">
+      <c r="C41" s="82" t="inlineStr">
         <is>
           <t>Mistake-proofing: the wrong action is blocked or corrected as it is attempted. Still durable, but it can be switched off, so name who owns the setting.</t>
         </is>
@@ -2044,7 +2047,7 @@
         <f>COUNTIF($P$10:$P$27,LEFT(A42,1)&amp;"*")</f>
         <v/>
       </c>
-      <c r="C42" s="81" t="inlineStr">
+      <c r="C42" s="82" t="inlineStr">
         <is>
           <t>The failure still happens and something catches it without anyone looking. Useful, but you are now managing defects rather than preventing them.</t>
         </is>
@@ -2060,7 +2063,7 @@
         <f>COUNTIF($P$10:$P$27,LEFT(A43,1)&amp;"*")</f>
         <v/>
       </c>
-      <c r="C43" s="81" t="inlineStr">
+      <c r="C43" s="82" t="inlineStr">
         <is>
           <t>Depends on a person remembering. Decays with every new hire and every busy week — count these honestly rather than relying on them.</t>
         </is>
@@ -2076,7 +2079,7 @@
         <f>COUNTIF($P$10:$P$27,LEFT(A44,1)&amp;"*")</f>
         <v/>
       </c>
-      <c r="C44" s="81" t="inlineStr">
+      <c r="C44" s="82" t="inlineStr">
         <is>
           <t>A briefing, a poster, a line in the wiki. Half-life measured in weeks. If most of your controls sit here, the process will drift back after handover.</t>
         </is>

</xml_diff>